<commit_message>
add: finished database mock-up and added sql database file structure
</commit_message>
<xml_diff>
--- a/docs/db/databse_structure.xlsx
+++ b/docs/db/databse_structure.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\habbo\Documents\Projets\budget_buddy\docs\db\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{BB03F805-D994-409C-88F7-90BB64FC6924}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{586EF3F7-2C23-4FB8-9BEA-8F2F208B7440}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13875" xr2:uid="{51FFE64F-0FD4-4554-A722-1623301F6E5B}"/>
   </bookViews>
   <sheets>
-    <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
+    <sheet name="db" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="23">
   <si>
     <t>users</t>
   </si>
@@ -87,6 +87,24 @@
   </si>
   <si>
     <t>boolean</t>
+  </si>
+  <si>
+    <t>transactions</t>
+  </si>
+  <si>
+    <t>id_account</t>
+  </si>
+  <si>
+    <t>amount</t>
+  </si>
+  <si>
+    <t>type</t>
+  </si>
+  <si>
+    <t>date</t>
+  </si>
+  <si>
+    <t>&lt; 0 for withdrawal, &gt; 0 for deposit</t>
   </si>
 </sst>
 </file>
@@ -110,7 +128,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -133,20 +151,188 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -482,104 +668,170 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{65711E94-4E45-4E92-A983-67341C86A63D}">
-  <dimension ref="B3:G10"/>
+  <dimension ref="B2:G16"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
+    <col min="2" max="2" width="9.59765625" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="10.73046875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.46484375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.53125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="11.46484375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
+    <row r="2" spans="2:7" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
     <row r="3" spans="2:7" x14ac:dyDescent="0.45">
-      <c r="B3" s="1" t="s">
+      <c r="B3" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="1"/>
-      <c r="D3" s="1"/>
-      <c r="E3" s="1"/>
-      <c r="F3" s="1"/>
-      <c r="G3" s="1"/>
+      <c r="C3" s="12"/>
+      <c r="D3" s="12"/>
+      <c r="E3" s="12"/>
+      <c r="F3" s="12"/>
+      <c r="G3" s="13"/>
     </row>
     <row r="4" spans="2:7" x14ac:dyDescent="0.45">
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="14" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="D4" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="E4" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="F4" s="2" t="s">
+      <c r="F4" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="G4" s="3" t="s">
+      <c r="G4" s="15" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="2:7" x14ac:dyDescent="0.45">
-      <c r="B5" s="2" t="s">
+    <row r="5" spans="2:7" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="B5" s="16" t="s">
         <v>10</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="C5" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="D5" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="E5" s="2" t="s">
+      <c r="E5" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="F5" s="2" t="s">
+      <c r="F5" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="G5" s="3" t="s">
+      <c r="G5" s="18" t="s">
         <v>8</v>
       </c>
     </row>
+    <row r="7" spans="2:7" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
     <row r="8" spans="2:7" x14ac:dyDescent="0.45">
-      <c r="B8" t="s">
+      <c r="B8" s="3" t="s">
         <v>9</v>
       </c>
+      <c r="C8" s="4"/>
+      <c r="D8" s="4"/>
+      <c r="E8" s="4"/>
+      <c r="F8" s="5"/>
     </row>
     <row r="9" spans="2:7" x14ac:dyDescent="0.45">
-      <c r="B9" t="s">
+      <c r="B9" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="C9" t="s">
+      <c r="C9" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="D9" t="s">
+      <c r="D9" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="E9" t="s">
+      <c r="E9" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="F9" t="s">
+      <c r="F9" s="7" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="10" spans="2:7" x14ac:dyDescent="0.45">
-      <c r="B10" t="s">
+    <row r="10" spans="2:7" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="B10" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="C10" t="s">
+      <c r="C10" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="D10" t="s">
+      <c r="D10" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="E10" t="s">
+      <c r="E10" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="F10" t="s">
+      <c r="F10" s="10" t="s">
         <v>16</v>
       </c>
     </row>
+    <row r="12" spans="2:7" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
+    <row r="13" spans="2:7" x14ac:dyDescent="0.45">
+      <c r="B13" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C13" s="4"/>
+      <c r="D13" s="4"/>
+      <c r="E13" s="4"/>
+      <c r="F13" s="5"/>
+    </row>
+    <row r="14" spans="2:7" x14ac:dyDescent="0.45">
+      <c r="B14" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F14" s="7" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="15" spans="2:7" x14ac:dyDescent="0.45">
+      <c r="B15" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F15" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="16" spans="2:7" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="B16" s="8"/>
+      <c r="C16" s="19" t="s">
+        <v>22</v>
+      </c>
+      <c r="D16" s="19"/>
+      <c r="E16" s="19"/>
+      <c r="F16" s="10"/>
+    </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="4">
     <mergeCell ref="B3:G3"/>
+    <mergeCell ref="B8:F8"/>
+    <mergeCell ref="C16:E16"/>
+    <mergeCell ref="B13:F13"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
fix: updated db to include a description for transactions
</commit_message>
<xml_diff>
--- a/docs/db/databse_structure.xlsx
+++ b/docs/db/databse_structure.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\habbo\Documents\Projets\budget_buddy\docs\db\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{586EF3F7-2C23-4FB8-9BEA-8F2F208B7440}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2302734-81AC-49A9-84B1-B1E8F416D49F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13875" xr2:uid="{51FFE64F-0FD4-4554-A722-1623301F6E5B}"/>
+    <workbookView xWindow="2190" yWindow="1860" windowWidth="16200" windowHeight="9982" xr2:uid="{51FFE64F-0FD4-4554-A722-1623301F6E5B}"/>
   </bookViews>
   <sheets>
     <sheet name="db" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="24">
   <si>
     <t>users</t>
   </si>
@@ -105,6 +105,9 @@
   </si>
   <si>
     <t>&lt; 0 for withdrawal, &gt; 0 for deposit</t>
+  </si>
+  <si>
+    <t>description</t>
   </si>
 </sst>
 </file>
@@ -275,7 +278,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -283,15 +286,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -306,6 +300,21 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -316,24 +325,22 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -680,17 +687,17 @@
   <sheetData>
     <row r="2" spans="2:7" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
     <row r="3" spans="2:7" x14ac:dyDescent="0.45">
-      <c r="B3" s="11" t="s">
+      <c r="B3" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="12"/>
-      <c r="D3" s="12"/>
-      <c r="E3" s="12"/>
-      <c r="F3" s="12"/>
-      <c r="G3" s="13"/>
+      <c r="C3" s="14"/>
+      <c r="D3" s="14"/>
+      <c r="E3" s="14"/>
+      <c r="F3" s="14"/>
+      <c r="G3" s="15"/>
     </row>
     <row r="4" spans="2:7" x14ac:dyDescent="0.45">
-      <c r="B4" s="14" t="s">
+      <c r="B4" s="8" t="s">
         <v>1</v>
       </c>
       <c r="C4" s="1" t="s">
@@ -705,42 +712,42 @@
       <c r="F4" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="G4" s="15" t="s">
+      <c r="G4" s="9" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="5" spans="2:7" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B5" s="16" t="s">
+      <c r="B5" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="C5" s="17" t="s">
+      <c r="C5" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="D5" s="17" t="s">
+      <c r="D5" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="E5" s="17" t="s">
+      <c r="E5" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="F5" s="17" t="s">
+      <c r="F5" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="G5" s="18" t="s">
+      <c r="G5" s="12" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="7" spans="2:7" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
     <row r="8" spans="2:7" x14ac:dyDescent="0.45">
-      <c r="B8" s="3" t="s">
+      <c r="B8" s="16" t="s">
         <v>9</v>
       </c>
-      <c r="C8" s="4"/>
-      <c r="D8" s="4"/>
-      <c r="E8" s="4"/>
-      <c r="F8" s="5"/>
+      <c r="C8" s="17"/>
+      <c r="D8" s="17"/>
+      <c r="E8" s="17"/>
+      <c r="F8" s="18"/>
     </row>
     <row r="9" spans="2:7" x14ac:dyDescent="0.45">
-      <c r="B9" s="6" t="s">
+      <c r="B9" s="3" t="s">
         <v>1</v>
       </c>
       <c r="C9" s="2" t="s">
@@ -752,39 +759,40 @@
       <c r="E9" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="F9" s="7" t="s">
+      <c r="F9" s="4" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="10" spans="2:7" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B10" s="8" t="s">
+      <c r="B10" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="C10" s="9" t="s">
+      <c r="C10" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="D10" s="9" t="s">
+      <c r="D10" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="E10" s="9" t="s">
+      <c r="E10" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="F10" s="10" t="s">
+      <c r="F10" s="7" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="12" spans="2:7" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
     <row r="13" spans="2:7" x14ac:dyDescent="0.45">
-      <c r="B13" s="3" t="s">
+      <c r="B13" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="C13" s="4"/>
-      <c r="D13" s="4"/>
-      <c r="E13" s="4"/>
-      <c r="F13" s="5"/>
+      <c r="C13" s="17"/>
+      <c r="D13" s="17"/>
+      <c r="E13" s="17"/>
+      <c r="F13" s="17"/>
+      <c r="G13" s="18"/>
     </row>
     <row r="14" spans="2:7" x14ac:dyDescent="0.45">
-      <c r="B14" s="6" t="s">
+      <c r="B14" s="3" t="s">
         <v>1</v>
       </c>
       <c r="C14" s="2" t="s">
@@ -796,12 +804,15 @@
       <c r="E14" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="F14" s="7" t="s">
+      <c r="F14" s="2" t="s">
         <v>21</v>
       </c>
+      <c r="G14" s="20" t="s">
+        <v>23</v>
+      </c>
     </row>
     <row r="15" spans="2:7" x14ac:dyDescent="0.45">
-      <c r="B15" s="6" t="s">
+      <c r="B15" s="3" t="s">
         <v>10</v>
       </c>
       <c r="C15" s="2" t="s">
@@ -813,25 +824,29 @@
       <c r="E15" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F15" s="7" t="s">
+      <c r="F15" s="2" t="s">
         <v>8</v>
       </c>
+      <c r="G15" s="20" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="16" spans="2:7" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B16" s="8"/>
+      <c r="B16" s="5"/>
       <c r="C16" s="19" t="s">
         <v>22</v>
       </c>
       <c r="D16" s="19"/>
       <c r="E16" s="19"/>
-      <c r="F16" s="10"/>
+      <c r="F16" s="6"/>
+      <c r="G16" s="21"/>
     </row>
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="B3:G3"/>
     <mergeCell ref="B8:F8"/>
     <mergeCell ref="C16:E16"/>
-    <mergeCell ref="B13:F13"/>
+    <mergeCell ref="B13:G13"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>